<commit_message>
actualización sección de políticas
</commit_message>
<xml_diff>
--- a/ejes/Políticas/Configuracion_politicas_bienestar.xlsx
+++ b/ejes/Políticas/Configuracion_politicas_bienestar.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -540,6 +540,35 @@
       <c r="C5" t="inlineStr">
         <is>
           <t>Instrucción directa de Felipe (2026-05-21): descartar esta política del repositorio, no listarla en Reporte a políticas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Negra, Afrocolombiana</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1.3.9</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Producto a nivel servicio Casas (no eje Bienestar). Ver Reporte a políticas en pagina principal de Casas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>PAD Víctimas</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Producto transversal a nivel servicio Casas (no eje Bienestar). Aplica a los 3 servicios.</t>
         </is>
       </c>
     </row>

</xml_diff>